<commit_message>
CFD con rejillas apiladas verticalmente (disposición BRINSA): INF-001 actualizado con 8 figuras y análisis reescrito; HD-REJ-001, dashboard y bases de diseño propagados; 7 entregables re-emitidos
</commit_message>
<xml_diff>
--- a/Emisiones/3.0 HV-HOJAS DE DATOS/P2437-HV-DTS-003.xlsx
+++ b/Emisiones/3.0 HV-HOJAS DE DATOS/P2437-HV-DTS-003.xlsx
@@ -3708,7 +3708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3727,8 +3727,7 @@
     <col width="35" customWidth="1" min="14" max="14"/>
     <col width="35" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="13" customWidth="1" min="25" max="25"/>
@@ -3736,8 +3735,8 @@
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="13" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
-    <col width="13" customWidth="1" min="33" max="33"/>
-    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
     <col width="13" customWidth="1" min="36" max="36"/>
     <col width="13" customWidth="1" min="37" max="37"/>
     <col width="13" customWidth="1" min="38" max="38"/>
@@ -3747,15 +3746,16 @@
     <col width="13" customWidth="1" min="42" max="42"/>
     <col width="13" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
-    <col width="13" customWidth="1" min="48" max="48"/>
-    <col width="13" customWidth="1" min="50" max="50"/>
+    <col width="13" customWidth="1" min="45" max="45"/>
+    <col width="13" customWidth="1" min="49" max="49"/>
     <col width="13" customWidth="1" min="51" max="51"/>
     <col width="13" customWidth="1" min="52" max="52"/>
     <col width="13" customWidth="1" min="53" max="53"/>
     <col width="13" customWidth="1" min="54" max="54"/>
     <col width="13" customWidth="1" min="55" max="55"/>
-    <col width="13" customWidth="1" min="57" max="57"/>
-    <col width="13" customWidth="1" min="62" max="62"/>
+    <col width="13" customWidth="1" min="56" max="56"/>
+    <col width="13" customWidth="1" min="58" max="58"/>
+    <col width="13" customWidth="1" min="63" max="63"/>
   </cols>
   <sheetData>
     <row r="1" ht="29.25" customHeight="1">
@@ -4037,7 +4037,7 @@
       <c r="H12" s="84" t="n"/>
       <c r="I12" s="83" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J12" s="84" t="n"/>
@@ -4137,75 +4137,57 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="50" customHeight="1"/>
-    <row r="20" ht="150" customHeight="1">
-      <c r="A20" s="81" t="inlineStr">
+    <row r="19" ht="700" customHeight="1">
+      <c r="A19" s="85" t="inlineStr">
+        <is>
+          <t>1.2. Disposición: las tres rejillas se instalan apiladas verticalmente, una sobre otra, en la pared opuesta a la inyección del ventilador, conforme a la disposición definida por BRINSA. Esta configuración fue validada mediante el modelo CFD del recinto: el chorro de inyección alimenta directamente la rejilla central y las recirculaciones superior e inferior distribuyen el caudal hacia las rejillas de los extremos, con velocidades faciales del orden de 3 m/s en los tres niveles (ver P2437-HV-INF-001, sección de resultados CFD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1"/>
+    <row r="21" ht="150" customHeight="1">
+      <c r="A21" s="81" t="inlineStr">
         <is>
           <t>2. Condiciones de operación y desempeño</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="100" customHeight="1">
-      <c r="A21" s="86" t="inlineStr">
+    <row r="22" ht="100" customHeight="1">
+      <c r="A22" s="86" t="inlineStr">
         <is>
           <t>Tabla 1. Condiciones de diseño (valores congelados de la memoria de cálculo).</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="50" customHeight="1">
-      <c r="A22" s="82" t="inlineStr">
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="82" t="inlineStr">
         <is>
           <t>Parámetro</t>
         </is>
       </c>
-      <c r="B22" s="82" t="n"/>
-      <c r="C22" s="82" t="n"/>
-      <c r="D22" s="82" t="n"/>
-      <c r="E22" s="82" t="n"/>
-      <c r="F22" s="82" t="n"/>
-      <c r="G22" s="82" t="n"/>
-      <c r="H22" s="82" t="n"/>
-      <c r="I22" s="82" t="inlineStr">
+      <c r="B23" s="82" t="n"/>
+      <c r="C23" s="82" t="n"/>
+      <c r="D23" s="82" t="n"/>
+      <c r="E23" s="82" t="n"/>
+      <c r="F23" s="82" t="n"/>
+      <c r="G23" s="82" t="n"/>
+      <c r="H23" s="82" t="n"/>
+      <c r="I23" s="82" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="J22" s="82" t="n"/>
-      <c r="K22" s="82" t="n"/>
-      <c r="L22" s="82" t="n"/>
-      <c r="M22" s="82" t="n"/>
-      <c r="N22" s="82" t="n"/>
-      <c r="O22" s="82" t="n"/>
-    </row>
-    <row r="23" ht="50" customHeight="1">
-      <c r="A23" s="83" t="inlineStr">
+      <c r="J23" s="82" t="n"/>
+      <c r="K23" s="82" t="n"/>
+      <c r="L23" s="82" t="n"/>
+      <c r="M23" s="82" t="n"/>
+      <c r="N23" s="82" t="n"/>
+      <c r="O23" s="82" t="n"/>
+    </row>
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="83" t="inlineStr">
         <is>
           <t>Cantidad</t>
-        </is>
-      </c>
-      <c r="B23" s="84" t="n"/>
-      <c r="C23" s="84" t="n"/>
-      <c r="D23" s="84" t="n"/>
-      <c r="E23" s="84" t="n"/>
-      <c r="F23" s="84" t="n"/>
-      <c r="G23" s="84" t="n"/>
-      <c r="H23" s="84" t="n"/>
-      <c r="I23" s="83" t="inlineStr">
-        <is>
-          <t>3 unidades</t>
-        </is>
-      </c>
-      <c r="J23" s="84" t="n"/>
-      <c r="K23" s="84" t="n"/>
-      <c r="L23" s="84" t="n"/>
-      <c r="M23" s="84" t="n"/>
-      <c r="N23" s="84" t="n"/>
-      <c r="O23" s="84" t="n"/>
-    </row>
-    <row r="24" ht="150" customHeight="1">
-      <c r="A24" s="83" t="inlineStr">
-        <is>
-          <t>Dimensiones faciales (unitarias)</t>
         </is>
       </c>
       <c r="B24" s="84" t="n"/>
@@ -4217,7 +4199,7 @@
       <c r="H24" s="84" t="n"/>
       <c r="I24" s="83" t="inlineStr">
         <is>
-          <t>353×336 mm (área facial 0.1187 m²)</t>
+          <t>3 unidades</t>
         </is>
       </c>
       <c r="J24" s="84" t="n"/>
@@ -4227,10 +4209,10 @@
       <c r="N24" s="84" t="n"/>
       <c r="O24" s="84" t="n"/>
     </row>
-    <row r="25" ht="100" customHeight="1">
+    <row r="25" ht="150" customHeight="1">
       <c r="A25" s="83" t="inlineStr">
         <is>
-          <t>Caudal total de descarga</t>
+          <t>Dimensiones faciales (unitarias)</t>
         </is>
       </c>
       <c r="B25" s="84" t="n"/>
@@ -4242,7 +4224,7 @@
       <c r="H25" s="84" t="n"/>
       <c r="I25" s="83" t="inlineStr">
         <is>
-          <t>3 840 m³/h (1.0667 m³/s)</t>
+          <t>353×336 mm (área facial 0.1187 m²)</t>
         </is>
       </c>
       <c r="J25" s="84" t="n"/>
@@ -4255,7 +4237,7 @@
     <row r="26" ht="100" customHeight="1">
       <c r="A26" s="83" t="inlineStr">
         <is>
-          <t>Velocidad facial</t>
+          <t>Caudal total de descarga</t>
         </is>
       </c>
       <c r="B26" s="84" t="n"/>
@@ -4267,7 +4249,7 @@
       <c r="H26" s="84" t="n"/>
       <c r="I26" s="83" t="inlineStr">
         <is>
-          <t>3 m/s</t>
+          <t>3 840 m³/h (1.0667 m³/s)</t>
         </is>
       </c>
       <c r="J26" s="84" t="n"/>
@@ -4277,10 +4259,10 @@
       <c r="N26" s="84" t="n"/>
       <c r="O26" s="84" t="n"/>
     </row>
-    <row r="27" ht="200" customHeight="1">
+    <row r="27" ht="100" customHeight="1">
       <c r="A27" s="83" t="inlineStr">
         <is>
-          <t>ΔP unitaria (cierre de orificio, C_d = 0.60, en el sitio)</t>
+          <t>Velocidad facial</t>
         </is>
       </c>
       <c r="B27" s="84" t="n"/>
@@ -4292,7 +4274,7 @@
       <c r="H27" s="84" t="n"/>
       <c r="I27" s="83" t="inlineStr">
         <is>
-          <t>11 Pa</t>
+          <t>3 m/s</t>
         </is>
       </c>
       <c r="J27" s="84" t="n"/>
@@ -4305,7 +4287,7 @@
     <row r="28" ht="200" customHeight="1">
       <c r="A28" s="83" t="inlineStr">
         <is>
-          <t>ΔP equivalente a densidad estándar (ρ = 1.2 kg/m³)</t>
+          <t>ΔP unitaria (cierre de orificio, C_d = 0.60, en el sitio)</t>
         </is>
       </c>
       <c r="B28" s="84" t="n"/>
@@ -4317,7 +4299,7 @@
       <c r="H28" s="84" t="n"/>
       <c r="I28" s="83" t="inlineStr">
         <is>
-          <t>15 Pa</t>
+          <t>11 Pa</t>
         </is>
       </c>
       <c r="J28" s="84" t="n"/>
@@ -4327,10 +4309,10 @@
       <c r="N28" s="84" t="n"/>
       <c r="O28" s="84" t="n"/>
     </row>
-    <row r="29" ht="150" customHeight="1">
+    <row r="29" ht="200" customHeight="1">
       <c r="A29" s="83" t="inlineStr">
         <is>
-          <t>Densidad del aire de diseño</t>
+          <t>ΔP equivalente a densidad estándar (ρ = 1.2 kg/m³)</t>
         </is>
       </c>
       <c r="B29" s="84" t="n"/>
@@ -4342,7 +4324,7 @@
       <c r="H29" s="84" t="n"/>
       <c r="I29" s="83" t="inlineStr">
         <is>
-          <t>0.88 kg/m³ (2 558 msnm, 74.1 kPa)</t>
+          <t>15 Pa</t>
         </is>
       </c>
       <c r="J29" s="84" t="n"/>
@@ -4352,83 +4334,83 @@
       <c r="N29" s="84" t="n"/>
       <c r="O29" s="84" t="n"/>
     </row>
-    <row r="30" ht="50" customHeight="1"/>
-    <row r="31" ht="400" customHeight="1">
-      <c r="A31" s="85" t="inlineStr">
+    <row r="30" ht="150" customHeight="1">
+      <c r="A30" s="83" t="inlineStr">
+        <is>
+          <t>Densidad del aire de diseño</t>
+        </is>
+      </c>
+      <c r="B30" s="84" t="n"/>
+      <c r="C30" s="84" t="n"/>
+      <c r="D30" s="84" t="n"/>
+      <c r="E30" s="84" t="n"/>
+      <c r="F30" s="84" t="n"/>
+      <c r="G30" s="84" t="n"/>
+      <c r="H30" s="84" t="n"/>
+      <c r="I30" s="83" t="inlineStr">
+        <is>
+          <t>0.88 kg/m³ (2 558 msnm, 74.1 kPa)</t>
+        </is>
+      </c>
+      <c r="J30" s="84" t="n"/>
+      <c r="K30" s="84" t="n"/>
+      <c r="L30" s="84" t="n"/>
+      <c r="M30" s="84" t="n"/>
+      <c r="N30" s="84" t="n"/>
+      <c r="O30" s="84" t="n"/>
+    </row>
+    <row r="31" ht="50" customHeight="1"/>
+    <row r="32" ht="400" customHeight="1">
+      <c r="A32" s="85" t="inlineStr">
         <is>
           <t>2.1. Nota de contexto: la ΔP unitaria de 11 Pa (cierre de orificio, C_d = 0.60, a 3 m/s) es la pérdida de descarga libre a la atmósfera y se suma a la caída de presión de la etapa filtrante para definir el punto de trabajo del ventilador; no existe consigna de presión interior que sostener.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="50" customHeight="1"/>
-    <row r="33" ht="150" customHeight="1">
-      <c r="A33" s="81" t="inlineStr">
+    <row r="33" ht="50" customHeight="1"/>
+    <row r="34" ht="150" customHeight="1">
+      <c r="A34" s="81" t="inlineStr">
         <is>
           <t>3. Construcción y áreas netas</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="50" customHeight="1">
-      <c r="A34" s="86" t="inlineStr">
+    <row r="35" ht="50" customHeight="1">
+      <c r="A35" s="86" t="inlineStr">
         <is>
           <t>Tabla 2. Especificación constructiva.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="50" customHeight="1">
-      <c r="A35" s="82" t="inlineStr">
+    <row r="36" ht="50" customHeight="1">
+      <c r="A36" s="82" t="inlineStr">
         <is>
           <t>Característica</t>
         </is>
       </c>
-      <c r="B35" s="82" t="n"/>
-      <c r="C35" s="82" t="n"/>
-      <c r="D35" s="82" t="n"/>
-      <c r="E35" s="82" t="n"/>
-      <c r="F35" s="82" t="n"/>
-      <c r="G35" s="82" t="n"/>
-      <c r="H35" s="82" t="n"/>
-      <c r="I35" s="82" t="inlineStr">
+      <c r="B36" s="82" t="n"/>
+      <c r="C36" s="82" t="n"/>
+      <c r="D36" s="82" t="n"/>
+      <c r="E36" s="82" t="n"/>
+      <c r="F36" s="82" t="n"/>
+      <c r="G36" s="82" t="n"/>
+      <c r="H36" s="82" t="n"/>
+      <c r="I36" s="82" t="inlineStr">
         <is>
           <t>Especificación</t>
         </is>
       </c>
-      <c r="J35" s="82" t="n"/>
-      <c r="K35" s="82" t="n"/>
-      <c r="L35" s="82" t="n"/>
-      <c r="M35" s="82" t="n"/>
-      <c r="N35" s="82" t="n"/>
-      <c r="O35" s="82" t="n"/>
-    </row>
-    <row r="36" ht="200" customHeight="1">
-      <c r="A36" s="83" t="inlineStr">
+      <c r="J36" s="82" t="n"/>
+      <c r="K36" s="82" t="n"/>
+      <c r="L36" s="82" t="n"/>
+      <c r="M36" s="82" t="n"/>
+      <c r="N36" s="82" t="n"/>
+      <c r="O36" s="82" t="n"/>
+    </row>
+    <row r="37" ht="200" customHeight="1">
+      <c r="A37" s="83" t="inlineStr">
         <is>
           <t>Tipo de núcleo</t>
-        </is>
-      </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="83" t="inlineStr">
-        <is>
-          <t>Eggcrate (panal) ½×½×½ in (12.7 mm), máxima área libre</t>
-        </is>
-      </c>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
-      <c r="L36" s="84" t="n"/>
-      <c r="M36" s="84" t="n"/>
-      <c r="N36" s="84" t="n"/>
-      <c r="O36" s="84" t="n"/>
-    </row>
-    <row r="37" ht="600" customHeight="1">
-      <c r="A37" s="83" t="inlineStr">
-        <is>
-          <t>Área libre del núcleo</t>
         </is>
       </c>
       <c r="B37" s="84" t="n"/>
@@ -4440,7 +4422,7 @@
       <c r="H37" s="84" t="n"/>
       <c r="I37" s="83" t="inlineStr">
         <is>
-          <t>≥ 90 % (cifra repetida en catálogos del tipo; Airfoil RC-FCR5 (https://airfoil.com.au/product/removable-core-fixing-clip-eggcrate-grille-rc-fcr5/), consulta 2026-07-23)</t>
+          <t>Eggcrate (panal) ½×½×½ in (12.7 mm), máxima área libre</t>
         </is>
       </c>
       <c r="J37" s="84" t="n"/>
@@ -4450,10 +4432,10 @@
       <c r="N37" s="84" t="n"/>
       <c r="O37" s="84" t="n"/>
     </row>
-    <row r="38" ht="950" customHeight="1">
+    <row r="38" ht="600" customHeight="1">
       <c r="A38" s="83" t="inlineStr">
         <is>
-          <t>Malla anti-insectos</t>
+          <t>Área libre del núcleo</t>
         </is>
       </c>
       <c r="B38" s="84" t="n"/>
@@ -4465,7 +4447,7 @@
       <c r="H38" s="84" t="n"/>
       <c r="I38" s="83" t="inlineStr">
         <is>
-          <t>Tejido 18×18, abertura ≈1 mm, alambre 0.45 mm, área abierta ≥ 48 % (tabla Industrial Metal Mesh (https://www.industrialmetalmesh.com/sale-54819921-micron-304-316l-stainless-steel-wire-mesh-screen-filter-mesh.html), consulta 2026-07-23); excluye insectos comunes</t>
+          <t>≥ 90 % (cifra repetida en catálogos del tipo; Airfoil RC-FCR5 (https://airfoil.com.au/product/removable-core-fixing-clip-eggcrate-grille-rc-fcr5/), consulta 2026-07-23)</t>
         </is>
       </c>
       <c r="J38" s="84" t="n"/>
@@ -4475,10 +4457,10 @@
       <c r="N38" s="84" t="n"/>
       <c r="O38" s="84" t="n"/>
     </row>
-    <row r="39" ht="200" customHeight="1">
+    <row r="39" ht="950" customHeight="1">
       <c r="A39" s="83" t="inlineStr">
         <is>
-          <t>Área neta combinada (núcleo + malla)</t>
+          <t>Malla anti-insectos</t>
         </is>
       </c>
       <c r="B39" s="84" t="n"/>
@@ -4490,7 +4472,7 @@
       <c r="H39" s="84" t="n"/>
       <c r="I39" s="83" t="inlineStr">
         <is>
-          <t>≈ 45 % del área facial (dato típico: 0.90 × 0.50)</t>
+          <t>Tejido 18×18, abertura ≈1 mm, alambre 0.45 mm, área abierta ≥ 48 % (tabla Industrial Metal Mesh (https://www.industrialmetalmesh.com/sale-54819921-micron-304-316l-stainless-steel-wire-mesh-screen-filter-mesh.html), consulta 2026-07-23); excluye insectos comunes</t>
         </is>
       </c>
       <c r="J39" s="84" t="n"/>
@@ -4500,10 +4482,10 @@
       <c r="N39" s="84" t="n"/>
       <c r="O39" s="84" t="n"/>
     </row>
-    <row r="40" ht="250" customHeight="1">
+    <row r="40" ht="200" customHeight="1">
       <c r="A40" s="83" t="inlineStr">
         <is>
-          <t>Material de la rejilla</t>
+          <t>Área neta combinada (núcleo + malla)</t>
         </is>
       </c>
       <c r="B40" s="84" t="n"/>
@@ -4515,7 +4497,7 @@
       <c r="H40" s="84" t="n"/>
       <c r="I40" s="83" t="inlineStr">
         <is>
-          <t>Inox 316L (primera opción) o aluminio anodizado 6063-T5 (alternativa)</t>
+          <t>≈ 45 % del área facial (dato típico: 0.90 × 0.50)</t>
         </is>
       </c>
       <c r="J40" s="84" t="n"/>
@@ -4525,10 +4507,10 @@
       <c r="N40" s="84" t="n"/>
       <c r="O40" s="84" t="n"/>
     </row>
-    <row r="41" ht="100" customHeight="1">
+    <row r="41" ht="250" customHeight="1">
       <c r="A41" s="83" t="inlineStr">
         <is>
-          <t>Material de la malla</t>
+          <t>Material de la rejilla</t>
         </is>
       </c>
       <c r="B41" s="84" t="n"/>
@@ -4540,7 +4522,7 @@
       <c r="H41" s="84" t="n"/>
       <c r="I41" s="83" t="inlineStr">
         <is>
-          <t>Inox 316</t>
+          <t>Inox 316L (primera opción) o aluminio anodizado 6063-T5 (alternativa)</t>
         </is>
       </c>
       <c r="J41" s="84" t="n"/>
@@ -4550,10 +4532,10 @@
       <c r="N41" s="84" t="n"/>
       <c r="O41" s="84" t="n"/>
     </row>
-    <row r="42" ht="150" customHeight="1">
+    <row r="42" ht="100" customHeight="1">
       <c r="A42" s="83" t="inlineStr">
         <is>
-          <t>Montaje de la malla</t>
+          <t>Material de la malla</t>
         </is>
       </c>
       <c r="B42" s="84" t="n"/>
@@ -4565,7 +4547,7 @@
       <c r="H42" s="84" t="n"/>
       <c r="I42" s="83" t="inlineStr">
         <is>
-          <t>Marco desmontable para limpieza periódica</t>
+          <t>Inox 316</t>
         </is>
       </c>
       <c r="J42" s="84" t="n"/>
@@ -4575,10 +4557,10 @@
       <c r="N42" s="84" t="n"/>
       <c r="O42" s="84" t="n"/>
     </row>
-    <row r="43" ht="350" customHeight="1">
+    <row r="43" ht="150" customHeight="1">
       <c r="A43" s="83" t="inlineStr">
         <is>
-          <t>Par galvánico</t>
+          <t>Montaje de la malla</t>
         </is>
       </c>
       <c r="B43" s="84" t="n"/>
@@ -4590,7 +4572,7 @@
       <c r="H43" s="84" t="n"/>
       <c r="I43" s="83" t="inlineStr">
         <is>
-          <t>Si se combina marco de aluminio con malla inox, aislamiento dieléctrico (dato típico de ingeniería)</t>
+          <t>Marco desmontable para limpieza periódica</t>
         </is>
       </c>
       <c r="J43" s="84" t="n"/>
@@ -4600,10 +4582,10 @@
       <c r="N43" s="84" t="n"/>
       <c r="O43" s="84" t="n"/>
     </row>
-    <row r="44" ht="150" customHeight="1">
+    <row r="44" ht="350" customHeight="1">
       <c r="A44" s="83" t="inlineStr">
         <is>
-          <t>Ensayo de desempeño</t>
+          <t>Par galvánico</t>
         </is>
       </c>
       <c r="B44" s="84" t="n"/>
@@ -4615,7 +4597,7 @@
       <c r="H44" s="84" t="n"/>
       <c r="I44" s="83" t="inlineStr">
         <is>
-          <t>ASHRAE 70 (medición de rejillas)</t>
+          <t>Si se combina marco de aluminio con malla inox, aislamiento dieléctrico (dato típico de ingeniería)</t>
         </is>
       </c>
       <c r="J44" s="84" t="n"/>
@@ -4625,135 +4607,123 @@
       <c r="N44" s="84" t="n"/>
       <c r="O44" s="84" t="n"/>
     </row>
-    <row r="45" ht="50" customHeight="1"/>
-    <row r="46" ht="350" customHeight="1">
-      <c r="A46" s="85" t="inlineStr">
+    <row r="45" ht="150" customHeight="1">
+      <c r="A45" s="83" t="inlineStr">
+        <is>
+          <t>Ensayo de desempeño</t>
+        </is>
+      </c>
+      <c r="B45" s="84" t="n"/>
+      <c r="C45" s="84" t="n"/>
+      <c r="D45" s="84" t="n"/>
+      <c r="E45" s="84" t="n"/>
+      <c r="F45" s="84" t="n"/>
+      <c r="G45" s="84" t="n"/>
+      <c r="H45" s="84" t="n"/>
+      <c r="I45" s="83" t="inlineStr">
+        <is>
+          <t>ASHRAE 70 (medición de rejillas)</t>
+        </is>
+      </c>
+      <c r="J45" s="84" t="n"/>
+      <c r="K45" s="84" t="n"/>
+      <c r="L45" s="84" t="n"/>
+      <c r="M45" s="84" t="n"/>
+      <c r="N45" s="84" t="n"/>
+      <c r="O45" s="84" t="n"/>
+    </row>
+    <row r="46" ht="50" customHeight="1"/>
+    <row r="47" ht="350" customHeight="1">
+      <c r="A47" s="85" t="inlineStr">
         <is>
           <t>3.1. La malla domina la pérdida del conjunto; el dimensionamiento por área neta combinada y la ΔP calculada por cierre de orificio (11 Pa) deben verificarse contra el área efectiva (Ak) del fabricante seleccionado (por confirmar con proveedor).</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="50" customHeight="1"/>
-    <row r="48" ht="100" customHeight="1">
-      <c r="A48" s="81" t="inlineStr">
+    <row r="48" ht="50" customHeight="1"/>
+    <row r="49" ht="100" customHeight="1">
+      <c r="A49" s="81" t="inlineStr">
         <is>
           <t>4. Candidatos comerciales</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="100" customHeight="1">
-      <c r="A49" s="86" t="inlineStr">
+    <row r="50" ht="100" customHeight="1">
+      <c r="A50" s="86" t="inlineStr">
         <is>
           <t>Tabla 3. Candidatos (consulta 2026-07-23).</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="100" customHeight="1">
-      <c r="A50" s="82" t="inlineStr">
+    <row r="51" ht="100" customHeight="1">
+      <c r="A51" s="82" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="B50" s="82" t="n"/>
-      <c r="C50" s="82" t="n"/>
-      <c r="D50" s="82" t="inlineStr">
+      <c r="B51" s="82" t="n"/>
+      <c r="C51" s="82" t="n"/>
+      <c r="D51" s="82" t="inlineStr">
         <is>
           <t>Tipo / material</t>
         </is>
       </c>
-      <c r="E50" s="82" t="n"/>
-      <c r="F50" s="82" t="n"/>
-      <c r="G50" s="82" t="inlineStr">
+      <c r="E51" s="82" t="n"/>
+      <c r="F51" s="82" t="n"/>
+      <c r="G51" s="82" t="inlineStr">
         <is>
           <t>Pros</t>
         </is>
       </c>
-      <c r="H50" s="82" t="n"/>
-      <c r="I50" s="82" t="n"/>
-      <c r="J50" s="82" t="inlineStr">
+      <c r="H51" s="82" t="n"/>
+      <c r="I51" s="82" t="n"/>
+      <c r="J51" s="82" t="inlineStr">
         <is>
           <t>Contras</t>
         </is>
       </c>
-      <c r="K50" s="82" t="n"/>
-      <c r="L50" s="82" t="n"/>
-      <c r="M50" s="82" t="inlineStr">
+      <c r="K51" s="82" t="n"/>
+      <c r="L51" s="82" t="n"/>
+      <c r="M51" s="82" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="N50" s="82" t="n"/>
-      <c r="O50" s="82" t="n"/>
-    </row>
-    <row r="51" ht="350" customHeight="1">
-      <c r="A51" s="83" t="inlineStr">
-        <is>
-          <t>Titus 50F / 50R</t>
-        </is>
-      </c>
-      <c r="B51" s="84" t="n"/>
-      <c r="C51" s="84" t="n"/>
-      <c r="D51" s="83" t="inlineStr">
-        <is>
-          <t>Eggcrate ½ in; aluminio, con versión íntegramente inox de fábrica</t>
-        </is>
-      </c>
-      <c r="E51" s="84" t="n"/>
-      <c r="F51" s="84" t="n"/>
-      <c r="G51" s="83" t="inlineStr">
-        <is>
-          <t>«Highest free area of any return grille»; única opción inox de catálogo</t>
-        </is>
-      </c>
-      <c r="H51" s="84" t="n"/>
-      <c r="I51" s="84" t="n"/>
-      <c r="J51" s="83" t="inlineStr">
-        <is>
-          <t>Importación; tamaño 353×336 por pedido</t>
-        </is>
-      </c>
-      <c r="K51" s="84" t="n"/>
-      <c r="L51" s="84" t="n"/>
-      <c r="M51" s="83" t="inlineStr">
-        <is>
-          <t>Titus 50F (PDF) (https://www.titus-hvac.com/file/1228/50F_50Rrprod_specialized_2017.pdf)</t>
-        </is>
-      </c>
-      <c r="N51" s="84" t="n"/>
-      <c r="O51" s="84" t="n"/>
+      <c r="N51" s="82" t="n"/>
+      <c r="O51" s="82" t="n"/>
     </row>
     <row r="52" ht="350" customHeight="1">
       <c r="A52" s="83" t="inlineStr">
         <is>
-          <t>Krueger EGC5</t>
+          <t>Titus 50F / 50R</t>
         </is>
       </c>
       <c r="B52" s="84" t="n"/>
       <c r="C52" s="84" t="n"/>
       <c r="D52" s="83" t="inlineStr">
         <is>
-          <t>Eggcrate ½ in; aluminio</t>
+          <t>Eggcrate ½ in; aluminio, con versión íntegramente inox de fábrica</t>
         </is>
       </c>
       <c r="E52" s="84" t="n"/>
       <c r="F52" s="84" t="n"/>
       <c r="G52" s="83" t="inlineStr">
         <is>
-          <t>Amplia gama de tamaños (6×4 in a 96×96 in)</t>
+          <t>«Highest free area of any return grille»; única opción inox de catálogo</t>
         </is>
       </c>
       <c r="H52" s="84" t="n"/>
       <c r="I52" s="84" t="n"/>
       <c r="J52" s="83" t="inlineStr">
         <is>
-          <t>Sin ejecución inox</t>
+          <t>Importación; tamaño 353×336 por pedido</t>
         </is>
       </c>
       <c r="K52" s="84" t="n"/>
       <c r="L52" s="84" t="n"/>
       <c r="M52" s="83" t="inlineStr">
         <is>
-          <t>Krueger EGC5 (https://www.krueger-hvac.com/Catalog%20Home/Grilles/Grilles%20-%20Return/EGC5)</t>
+          <t>Titus 50F (PDF) (https://www.titus-hvac.com/file/1228/50F_50Rrprod_specialized_2017.pdf)</t>
         </is>
       </c>
       <c r="N52" s="84" t="n"/>
@@ -4762,153 +4732,190 @@
     <row r="53" ht="350" customHeight="1">
       <c r="A53" s="83" t="inlineStr">
         <is>
-          <t>ProAire S.A.S (Bogotá)</t>
+          <t>Krueger EGC5</t>
         </is>
       </c>
       <c r="B53" s="84" t="n"/>
       <c r="C53" s="84" t="n"/>
       <c r="D53" s="83" t="inlineStr">
         <is>
-          <t>Fabricación a medida con corte láser, inox 316</t>
+          <t>Eggcrate ½ in; aluminio</t>
         </is>
       </c>
       <c r="E53" s="84" t="n"/>
       <c r="F53" s="84" t="n"/>
       <c r="G53" s="83" t="inlineStr">
         <is>
-          <t>Medida exacta 353×336 y ejecución inox 316L local; vía recomendada</t>
+          <t>Amplia gama de tamaños (6×4 in a 96×96 in)</t>
         </is>
       </c>
       <c r="H53" s="84" t="n"/>
       <c r="I53" s="84" t="n"/>
       <c r="J53" s="83" t="inlineStr">
         <is>
-          <t>Submittal y Ak por confirmar con proveedor</t>
+          <t>Sin ejecución inox</t>
         </is>
       </c>
       <c r="K53" s="84" t="n"/>
       <c r="L53" s="84" t="n"/>
       <c r="M53" s="83" t="inlineStr">
         <is>
-          <t>proairecolombia.com (https://www.proairecolombia.com/productos/rejillas-y-difusores.html)</t>
+          <t>Krueger EGC5 (https://www.krueger-hvac.com/Catalog%20Home/Grilles/Grilles%20-%20Return/EGC5)</t>
         </is>
       </c>
       <c r="N53" s="84" t="n"/>
       <c r="O53" s="84" t="n"/>
     </row>
-    <row r="54" ht="250" customHeight="1">
+    <row r="54" ht="350" customHeight="1">
       <c r="A54" s="83" t="inlineStr">
         <is>
-          <t>Laminaire (Colombia)</t>
+          <t>ProAire S.A.S (Bogotá)</t>
         </is>
       </c>
       <c r="B54" s="84" t="n"/>
       <c r="C54" s="84" t="n"/>
       <c r="D54" s="83" t="inlineStr">
         <is>
-          <t>Rejillas y difusores en aluminio a pedido</t>
+          <t>Fabricación a medida con corte láser, inox 316</t>
         </is>
       </c>
       <c r="E54" s="84" t="n"/>
       <c r="F54" s="84" t="n"/>
       <c r="G54" s="83" t="inlineStr">
         <is>
-          <t>Fabricación local con software de selección; marco para malla a pedido</t>
+          <t>Medida exacta 353×336 y ejecución inox 316L local; vía recomendada</t>
         </is>
       </c>
       <c r="H54" s="84" t="n"/>
       <c r="I54" s="84" t="n"/>
       <c r="J54" s="83" t="inlineStr">
         <is>
-          <t>Confirmar ejecución inox</t>
+          <t>Submittal y Ak por confirmar con proveedor</t>
         </is>
       </c>
       <c r="K54" s="84" t="n"/>
       <c r="L54" s="84" t="n"/>
       <c r="M54" s="83" t="inlineStr">
         <is>
-          <t>laminaire.net (https://laminaire.net/)</t>
+          <t>proairecolombia.com (https://www.proairecolombia.com/productos/rejillas-y-difusores.html)</t>
         </is>
       </c>
       <c r="N54" s="84" t="n"/>
       <c r="O54" s="84" t="n"/>
     </row>
-    <row r="55" ht="150" customHeight="1">
+    <row r="55" ht="250" customHeight="1">
       <c r="A55" s="83" t="inlineStr">
         <is>
-          <t>CL Ingeniería (Bogotá)</t>
+          <t>Laminaire (Colombia)</t>
         </is>
       </c>
       <c r="B55" s="84" t="n"/>
       <c r="C55" s="84" t="n"/>
       <c r="D55" s="83" t="inlineStr">
         <is>
-          <t>Rejillas y accesorios HVAC</t>
+          <t>Rejillas y difusores en aluminio a pedido</t>
         </is>
       </c>
       <c r="E55" s="84" t="n"/>
       <c r="F55" s="84" t="n"/>
       <c r="G55" s="83" t="inlineStr">
         <is>
-          <t>Canal local adicional</t>
+          <t>Fabricación local con software de selección; marco para malla a pedido</t>
         </is>
       </c>
       <c r="H55" s="84" t="n"/>
       <c r="I55" s="84" t="n"/>
       <c r="J55" s="83" t="inlineStr">
         <is>
-          <t>Catálogo genérico</t>
+          <t>Confirmar ejecución inox</t>
         </is>
       </c>
       <c r="K55" s="84" t="n"/>
       <c r="L55" s="84" t="n"/>
       <c r="M55" s="83" t="inlineStr">
         <is>
-          <t>clingenieria.co (https://clingenieria.co/)</t>
+          <t>laminaire.net (https://laminaire.net/)</t>
         </is>
       </c>
       <c r="N55" s="84" t="n"/>
       <c r="O55" s="84" t="n"/>
     </row>
-    <row r="56" ht="50" customHeight="1"/>
-    <row r="57" ht="50" customHeight="1">
-      <c r="A57" s="81" t="inlineStr">
+    <row r="56" ht="150" customHeight="1">
+      <c r="A56" s="83" t="inlineStr">
+        <is>
+          <t>CL Ingeniería (Bogotá)</t>
+        </is>
+      </c>
+      <c r="B56" s="84" t="n"/>
+      <c r="C56" s="84" t="n"/>
+      <c r="D56" s="83" t="inlineStr">
+        <is>
+          <t>Rejillas y accesorios HVAC</t>
+        </is>
+      </c>
+      <c r="E56" s="84" t="n"/>
+      <c r="F56" s="84" t="n"/>
+      <c r="G56" s="83" t="inlineStr">
+        <is>
+          <t>Canal local adicional</t>
+        </is>
+      </c>
+      <c r="H56" s="84" t="n"/>
+      <c r="I56" s="84" t="n"/>
+      <c r="J56" s="83" t="inlineStr">
+        <is>
+          <t>Catálogo genérico</t>
+        </is>
+      </c>
+      <c r="K56" s="84" t="n"/>
+      <c r="L56" s="84" t="n"/>
+      <c r="M56" s="83" t="inlineStr">
+        <is>
+          <t>clingenieria.co (https://clingenieria.co/)</t>
+        </is>
+      </c>
+      <c r="N56" s="84" t="n"/>
+      <c r="O56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="50" customHeight="1"/>
+    <row r="58" ht="50" customHeight="1">
+      <c r="A58" s="81" t="inlineStr">
         <is>
           <t>5. Instalación</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="450" customHeight="1">
-      <c r="A58" s="85" t="inlineStr">
+    <row r="59" ht="450" customHeight="1">
+      <c r="A59" s="85" t="inlineStr">
         <is>
           <t>5.1. Montaje a ras de muro exterior con marco perimetral sellado con silicona RTV neutra (compatible con hipoclorito; Chemical Resistance of RTV Silicone Sealants (PDF) (https://irp.cdn-website.com/63168859/files/uploaded/Chemical%20Resistance%20of%20RTV%20Silicone%20Sealants%20Chart.pdf), consulta 2026-07-23) y ferretería inox 316 (A4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="150" customHeight="1">
-      <c r="A59" s="85" t="inlineStr">
-        <is>
-          <t>5.2. Las bocas exteriores se orientan preferentemente a sotavento respecto de las fuentes de cloro de la planta.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="150" customHeight="1">
       <c r="A60" s="85" t="inlineStr">
         <is>
+          <t>5.2. Las bocas exteriores se orientan preferentemente a sotavento respecto de las fuentes de cloro de la planta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="150" customHeight="1">
+      <c r="A61" s="85" t="inlineStr">
+        <is>
           <t>5.3. Programa de limpieza de la malla según carga de polvo observada en comisionamiento (dato típico de operación).</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="50" customHeight="1"/>
-    <row r="62" ht="100" customHeight="1">
-      <c r="A62" s="81" t="inlineStr">
+    <row r="62" ht="50" customHeight="1"/>
+    <row r="63" ht="100" customHeight="1">
+      <c r="A63" s="81" t="inlineStr">
         <is>
           <t>6. Normas aplicables</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="500" customHeight="1">
-      <c r="A63" s="85" t="inlineStr">
+    <row r="64" ht="500" customHeight="1">
+      <c r="A64" s="85" t="inlineStr">
         <is>
           <t>6.1. ASHRAE 70 (método de ensayo y reporte de desempeño de rejillas); correlación de área libre para transferencia de aire según Building Science BA-0006 (https://buildingscience.com/sites/default/files/migrate/pdf/BA-0006_Discuss_transfer_grilles.pdf) (consulta 2026-07-23); ISO 12944 / NACE-AMPP para la selección de materiales en el ambiente clorado.</t>
         </is>
@@ -4920,13 +4927,13 @@
     <mergeCell ref="D53:F53"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="A25:H25"/>
-    <mergeCell ref="J50:L50"/>
+    <mergeCell ref="I30:O30"/>
     <mergeCell ref="N5:O5"/>
     <mergeCell ref="C2:L3"/>
     <mergeCell ref="A52:C52"/>
-    <mergeCell ref="G50:I50"/>
     <mergeCell ref="J52:L52"/>
     <mergeCell ref="M53:O53"/>
+    <mergeCell ref="A58:O58"/>
     <mergeCell ref="G52:I52"/>
     <mergeCell ref="I41:O41"/>
     <mergeCell ref="M55:O55"/>
@@ -4941,47 +4948,44 @@
     <mergeCell ref="A40:H40"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A24:H24"/>
-    <mergeCell ref="I35:O35"/>
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="I10:O10"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="G55:I55"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="G51:I51"/>
-    <mergeCell ref="A62:O62"/>
     <mergeCell ref="D55:F55"/>
     <mergeCell ref="I11:O11"/>
+    <mergeCell ref="I45:O45"/>
     <mergeCell ref="G54:I54"/>
-    <mergeCell ref="A20:O20"/>
     <mergeCell ref="D54:F54"/>
     <mergeCell ref="A42:H42"/>
-    <mergeCell ref="A48:O48"/>
-    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="M56:O56"/>
+    <mergeCell ref="G56:I56"/>
+    <mergeCell ref="A51:C51"/>
     <mergeCell ref="I28:O28"/>
-    <mergeCell ref="A51:C51"/>
     <mergeCell ref="I37:O37"/>
     <mergeCell ref="N6:O6"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="J53:L53"/>
     <mergeCell ref="I23:O23"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="G53:I53"/>
     <mergeCell ref="J55:L55"/>
-    <mergeCell ref="A50:C50"/>
     <mergeCell ref="J54:L54"/>
-    <mergeCell ref="A33:O33"/>
     <mergeCell ref="A41:H41"/>
+    <mergeCell ref="J56:L56"/>
     <mergeCell ref="A17:O17"/>
     <mergeCell ref="D51:F51"/>
     <mergeCell ref="I27:O27"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="I36:O36"/>
-    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="A63:O63"/>
+    <mergeCell ref="A34:O34"/>
+    <mergeCell ref="A9:O9"/>
     <mergeCell ref="A1:A5"/>
-    <mergeCell ref="A9:O9"/>
     <mergeCell ref="C1:L1"/>
-    <mergeCell ref="I22:O22"/>
-    <mergeCell ref="A35:H35"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="I12:O12"/>
     <mergeCell ref="M51:O51"/>
@@ -4990,13 +4994,16 @@
     <mergeCell ref="I14:O14"/>
     <mergeCell ref="I39:O39"/>
     <mergeCell ref="M54:O54"/>
+    <mergeCell ref="A56:C56"/>
     <mergeCell ref="I29:O29"/>
     <mergeCell ref="A36:H36"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="I38:O38"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A21:O21"/>
     <mergeCell ref="I13:O13"/>
-    <mergeCell ref="A57:O57"/>
     <mergeCell ref="I40:O40"/>
+    <mergeCell ref="D56:F56"/>
     <mergeCell ref="I15:O15"/>
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="A37:H37"/>
@@ -5004,12 +5011,12 @@
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="J51:L51"/>
     <mergeCell ref="I26:O26"/>
-    <mergeCell ref="M50:O50"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="I25:O25"/>
     <mergeCell ref="C4:L6"/>
     <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A49:O49"/>
     <mergeCell ref="D52:F52"/>
     <mergeCell ref="I42:O42"/>
   </mergeCells>

</xml_diff>